<commit_message>
Bar vendor list and drawing in metres
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plans/bar-boq.xlsx
+++ b/plans/bar-boq.xlsx
@@ -514,7 +514,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Shop 4, Tulip Residency, Gandaulim, Salcete, South Goa. Bar on the left wall as in the Simplex model. Grouped by area of the bar (A to H); the same letters and item numbers are on the A3 drawing. Sizes in mm (width × depth × height), the space available; measure on site.</t>
+          <t>Shop 4, Tulip Residency, Gandaulim, Salcete, South Goa. Bar on the left wall as in the Simplex model. Grouped by area of the bar (A to H); the same letters and item numbers are on the A3 drawing. Sizes in metres (width × depth × height), the space available; measure on site.</t>
         </is>
       </c>
     </row>
@@ -543,7 +543,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Size W × D × H (mm)</t>
+          <t>Size W × D × H (m)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -617,7 +617,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>2,200 × 750 × 1,040</t>
+          <t>2.20 × 0.75 × 1.04</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -651,13 +651,13 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>In front of the counter, 600 mm apart</t>
+          <t>In front of the counter, 0.60 m apart</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Seat height to suit the 1,040 mm counter</t>
+          <t>Seat height to suit the 1.04 m counter</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
@@ -691,12 +691,12 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>740 × 2,000</t>
+          <t>0.74 × 2.00</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Brass frame on 4 black rods; lower tier at 2,300 mm for stemware hung upside down, upper tier at 2,580 mm for pints and highballs; warm LED strips</t>
+          <t>Brass frame on 4 black rods; lower tier at 2.30 m for stemware hung upside down, upper tier at 2.58 m for pints and highballs; warm LED strips</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Ø 90 × 420 high</t>
+          <t>Ø 0.09 × 0.42 high</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>1,100 × 630 × 900</t>
+          <t>1.10 × 0.63 × 0.90</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Ø 240 × 420</t>
+          <t>Ø 0.24 × 0.42</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>500 × 420 × 570</t>
+          <t>0.50 × 0.42 × 0.57</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Ø 150 × 670</t>
+          <t>Ø 0.15 × 0.67</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>1,060 × 200 × 850</t>
+          <t>1.06 × 0.20 × 0.85</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1120,7 +1120,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>380 long</t>
+          <t>0.38 long</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>380 long</t>
+          <t>0.38 long</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>1,060 long</t>
+          <t>1.06 long</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>500 × 550 × 800</t>
+          <t>0.50 × 0.55 × 0.80</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1349,17 +1349,17 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Along the left wall, 2,650 mm long</t>
+          <t>Along the left wall, 2.65 m long</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>2,650 × 400 × 960</t>
+          <t>2.65 × 0.40 × 0.96</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Olive-wood doors and marble top; onyx panel from 960 to 2,380 mm with a sage panel above</t>
+          <t>Olive-wood doors and marble top; onyx panel from 0.96 to 2.38 m with a sage panel above</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -1393,12 +1393,12 @@
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>1,000 × 250</t>
+          <t>1.00 × 0.25</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Two brass-edged tiers at 1,300 and 1,740 mm; backlit onyx panel behind</t>
+          <t>Two brass-edged tiers at 1.30 and 1.74 m; backlit onyx panel behind</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -1432,12 +1432,12 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>600 long × 220</t>
+          <t>0.60 long × 0.22</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Glass shelf at 960 mm with 3 jars</t>
+          <t>Glass shelf at 0.96 m with 3 jars</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>1,140 × 620</t>
+          <t>1.14 × 0.62</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr"/>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>900 × 200</t>
+          <t>0.90 × 0.20</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr"/>
@@ -1614,17 +1614,17 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Part of the back bar, 550 mm deep here</t>
+          <t>Part of the back bar, 0.55 m deep here</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>1,270 × 550 × 960</t>
+          <t>1.27 × 0.55 × 0.96</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Bartender aisle is about 700 mm at this point</t>
+          <t>Bartender aisle is about 0.70 m at this point</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>450 × 500 × 820</t>
+          <t>0.45 × 0.50 × 0.82</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>700 × 520 × 860</t>
+          <t>0.70 × 0.52 × 0.86</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>480 × 400 × 960 to 1,350</t>
+          <t>0.48 × 0.40 × 0.96 to 1.35</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -1818,7 +1818,7 @@
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>400 × 240</t>
+          <t>0.40 × 0.24</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -1900,7 +1900,7 @@
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>800 × 500 × 940</t>
+          <t>0.80 × 0.50 × 0.94</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -1939,12 +1939,12 @@
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>800 × 300</t>
+          <t>0.80 × 0.30</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>At 1,600 and 1,950 mm, for glasses and cutlery</t>
+          <t>At 1.60 and 1.95 m, for glasses and cutlery</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Bar list: sink and ice well are one basin line (0.38 x 0.16 x 0.16 m)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plans/bar-boq.xlsx
+++ b/plans/bar-boq.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1049,14 +1049,14 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Bartender work area (sink, ice well, speed rail, ice machine)</t>
+          <t>Bartender work area (sink and ice basin, speed rail, ice machine)</t>
         </is>
       </c>
       <c r="C22" s="4" t="n"/>
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>The stainless area behind the counter at the far end, where the bartender washes, scoops ice and keeps the speed-rail bottles.</t>
+          <t>The stainless area behind the counter at the far end, where the bartender washes and scoops ice from the basin and keeps the speed-rail bottles.</t>
         </is>
       </c>
       <c r="F22" s="4" t="n"/>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Holds the next three items; one continuous stainless unit</t>
+          <t>Holds the sink basin and the speed rail below; one continuous stainless unit</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -1110,22 +1110,22 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Bar sink</t>
+          <t>Bar sink / ice well basin</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Set into the work unit</t>
+          <t>Set into the top of the work unit</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>0.38 long</t>
+          <t>0.38 × 0.16 × 0.16</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Hot and cold tap, drains to the grey-water line</t>
+          <t>One basin used for washing and as the ice well; hot and cold tap, drains to the grey-water line. The vendor may propose a deeper basin (then the unit depth changes)</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -1149,22 +1149,22 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Ice well</t>
+          <t>Speed rail</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Set into the work unit, beside the sink</t>
+          <t>Along the front of the work unit</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>0.38 long</t>
+          <t>1.06 long</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Insulated, with a drain</t>
+          <t>Holds the everyday spirit bottles within reach</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -1188,22 +1188,22 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Speed rail</t>
+          <t>Ice machine, under-counter</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Along the front of the work unit</t>
+          <t>Under the counter beside the work unit</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>1.06 long</t>
+          <t>0.50 × 0.55 × 0.80</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Holds the everyday spirit bottles within reach</t>
+          <t>About 50 kg a day; filtered cold water and a drain</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -1227,27 +1227,23 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Ice machine, under-counter</t>
+          <t>Water filter for the ice machine and the glasswasher</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Under the counter beside the work unit</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>0.50 × 0.55 × 0.80</t>
-        </is>
-      </c>
+          <t>Inside the cabinet next to the ice machine</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr"/>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>About 50 kg a day; filtered cold water and a drain</t>
+          <t>Cartridge type; replace on schedule</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>nos</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G27" s="6" t="n">
@@ -1261,82 +1257,86 @@
       <c r="J27" s="9" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="n">
+      <c r="A28" s="10" t="n"/>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Subtotal, section C</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="10" t="n"/>
+      <c r="H28" s="10" t="n"/>
+      <c r="I28" s="11">
+        <f>SUM(I23:I27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="10" t="n"/>
+    </row>
+    <row r="30" ht="46" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Back bar (the wall behind the bartender)</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n"/>
+      <c r="D30" s="4" t="n"/>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>The long unit along the left wall: cabinets below, display shelves and an onyx panel above.</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
+      <c r="I30" s="4" t="n"/>
+      <c r="J30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Water filter for the ice machine and the glasswasher</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Inside the cabinet next to the ice machine</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr"/>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>Cartridge type; replace on schedule</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>set</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H28" s="7" t="n"/>
-      <c r="I28" s="8">
-        <f>IF(H28="","",G28*H28)</f>
-        <v/>
-      </c>
-      <c r="J28" s="9" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="10" t="n"/>
-      <c r="B29" s="10" t="inlineStr">
-        <is>
-          <t>Subtotal, section C</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="n"/>
-      <c r="D29" s="10" t="n"/>
-      <c r="E29" s="10" t="n"/>
-      <c r="F29" s="10" t="n"/>
-      <c r="G29" s="10" t="n"/>
-      <c r="H29" s="10" t="n"/>
-      <c r="I29" s="11">
-        <f>SUM(I23:I28)</f>
-        <v/>
-      </c>
-      <c r="J29" s="10" t="n"/>
-    </row>
-    <row r="31" ht="46" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Back bar (the wall behind the bartender)</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>The long unit along the left wall: cabinets below, display shelves and an onyx panel above.</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="n"/>
-      <c r="G31" s="4" t="n"/>
-      <c r="H31" s="4" t="n"/>
-      <c r="I31" s="4" t="n"/>
-      <c r="J31" s="4" t="n"/>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Back bar run</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Along the left wall, 2.65 m long</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>2.65 × 0.40 × 0.96</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Olive-wood doors and marble top; onyx panel from 0.96 to 2.38 m with a sage panel above</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="H31" s="7" t="n"/>
+      <c r="I31" s="8">
+        <f>IF(H31="","",G31*H31)</f>
+        <v/>
+      </c>
+      <c r="J31" s="9" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="n">
@@ -1344,31 +1344,31 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Back bar run</t>
+          <t>Display shelves for whisky, gin and vodka</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Along the left wall, 2.65 m long</t>
+          <t>On the wall above the back bar</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>2.65 × 0.40 × 0.96</t>
+          <t>1.00 × 0.25</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Olive-wood doors and marble top; onyx panel from 0.96 to 2.38 m with a sage panel above</t>
+          <t>Two brass-edged tiers at 1.30 and 1.74 m; backlit onyx panel behind</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G32" s="6" t="n">
-        <v>2.65</v>
+        <v>1</v>
       </c>
       <c r="H32" s="7" t="n"/>
       <c r="I32" s="8">
@@ -1383,22 +1383,22 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Display shelves for whisky, gin and vodka</t>
+          <t>Infusion jars with a glass shelf</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>On the wall above the back bar</t>
+          <t>Door end of the back bar</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>1.00 × 0.25</t>
+          <t>0.60 long × 0.22</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Two brass-edged tiers at 1.30 and 1.74 m; backlit onyx panel behind</t>
+          <t>Glass shelf at 0.96 m with 3 jars</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -1422,22 +1422,18 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Infusion jars with a glass shelf</t>
+          <t>Soju display and ON TAP board</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Door end of the back bar</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>0.60 long × 0.22</t>
-        </is>
-      </c>
+          <t>Far end of the back bar, by the pillar</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr"/>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Glass shelf at 0.96 m with 3 jars</t>
+          <t>Size by the contractor; not drawn in the model</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -1461,23 +1457,23 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Soju display and ON TAP board</t>
+          <t>Wall TV with bracket</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Far end of the back bar, by the pillar</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr"/>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Size by the contractor; not drawn in the model</t>
-        </is>
-      </c>
+          <t>On the wall above the back bar, door end</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>1.14 × 0.62</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr"/>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>nos</t>
         </is>
       </c>
       <c r="G35" s="6" t="n">
@@ -1496,23 +1492,23 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Wall TV with bracket</t>
+          <t>Neon sign "settle up here" and two red neon tubes</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>On the wall above the back bar, door end</t>
+          <t>Over the POS nook; tubes on the back bar wall</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>1.14 × 0.62</t>
+          <t>0.90 × 0.20</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr"/>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>nos</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G36" s="6" t="n">
@@ -1526,82 +1522,86 @@
       <c r="J36" s="9" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="n">
+      <c r="A37" s="10" t="n"/>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Subtotal, section D</t>
+        </is>
+      </c>
+      <c r="C37" s="10" t="n"/>
+      <c r="D37" s="10" t="n"/>
+      <c r="E37" s="10" t="n"/>
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="10" t="n"/>
+      <c r="H37" s="10" t="n"/>
+      <c r="I37" s="11">
+        <f>SUM(I31:I36)</f>
+        <v/>
+      </c>
+      <c r="J37" s="10" t="n"/>
+    </row>
+    <row r="39" ht="46" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Built-in section (glasswasher and drinks cooler)</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="n"/>
+      <c r="D39" s="4" t="n"/>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>A deeper stretch of the back bar opposite the bartender work area. The glasswasher and the cooler sit side by side in it.</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="n"/>
+      <c r="G39" s="4" t="n"/>
+      <c r="H39" s="4" t="n"/>
+      <c r="I39" s="4" t="n"/>
+      <c r="J39" s="4" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="n">
         <v>22</v>
       </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Neon sign "settle up here" and two red neon tubes</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Over the POS nook; tubes on the back bar wall</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>0.90 × 0.20</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr"/>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>set</t>
-        </is>
-      </c>
-      <c r="G37" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H37" s="7" t="n"/>
-      <c r="I37" s="8">
-        <f>IF(H37="","",G37*H37)</f>
-        <v/>
-      </c>
-      <c r="J37" s="9" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="10" t="n"/>
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>Subtotal, section D</t>
-        </is>
-      </c>
-      <c r="C38" s="10" t="n"/>
-      <c r="D38" s="10" t="n"/>
-      <c r="E38" s="10" t="n"/>
-      <c r="F38" s="10" t="n"/>
-      <c r="G38" s="10" t="n"/>
-      <c r="H38" s="10" t="n"/>
-      <c r="I38" s="11">
-        <f>SUM(I32:I37)</f>
-        <v/>
-      </c>
-      <c r="J38" s="10" t="n"/>
-    </row>
-    <row r="40" ht="46" customHeight="1">
-      <c r="A40" s="4" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Built-in section (glasswasher and drinks cooler)</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>A deeper stretch of the back bar opposite the bartender work area. The glasswasher and the cooler sit side by side in it.</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="n"/>
-      <c r="H40" s="4" t="n"/>
-      <c r="I40" s="4" t="n"/>
-      <c r="J40" s="4" t="n"/>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Built-in cabinet for the glasswasher and cooler</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Part of the back bar, 0.55 m deep here</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>1.27 × 0.55 × 0.96</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Bartender aisle is about 0.70 m at this point</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>nos</t>
+        </is>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="7" t="n"/>
+      <c r="I40" s="8">
+        <f>IF(H40="","",G40*H40)</f>
+        <v/>
+      </c>
+      <c r="J40" s="9" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="n">
@@ -1609,22 +1609,22 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Built-in cabinet for the glasswasher and cooler</t>
+          <t>Under-counter glasswasher</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Part of the back bar, 0.55 m deep here</t>
+          <t>In the built-in cabinet, toward the far end</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>1.27 × 0.55 × 0.96</t>
+          <t>0.45 × 0.50 × 0.82</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Bartender aisle is about 0.70 m at this point</t>
+          <t>Drop-down door; hot and cold water and a drain</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
@@ -1648,22 +1648,22 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Under-counter glasswasher</t>
+          <t>Glass-door drinks cooler</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>In the built-in cabinet, toward the far end</t>
+          <t>In the built-in cabinet, toward the door</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>0.45 × 0.50 × 0.82</t>
+          <t>0.70 × 0.52 × 0.86</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Drop-down door; hot and cold water and a drain</t>
+          <t>Lit; for mixers, water and soft drinks; state litres</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
@@ -1682,86 +1682,86 @@
       <c r="J42" s="9" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="n">
+      <c r="A43" s="10" t="n"/>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Subtotal, section E</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="n"/>
+      <c r="D43" s="10" t="n"/>
+      <c r="E43" s="10" t="n"/>
+      <c r="F43" s="10" t="n"/>
+      <c r="G43" s="10" t="n"/>
+      <c r="H43" s="10" t="n"/>
+      <c r="I43" s="11">
+        <f>SUM(I40:I42)</f>
+        <v/>
+      </c>
+      <c r="J43" s="10" t="n"/>
+    </row>
+    <row r="45" ht="46" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Cash and POS</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="n"/>
+      <c r="D45" s="4" t="n"/>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>At the door end of the back bar, where bills are settled.</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
+      <c r="H45" s="4" t="n"/>
+      <c r="I45" s="4" t="n"/>
+      <c r="J45" s="4" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>Glass-door drinks cooler</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>In the built-in cabinet, toward the door</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>0.70 × 0.52 × 0.86</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Lit; for mixers, water and soft drinks; state litres</t>
-        </is>
-      </c>
-      <c r="F43" s="5" t="inlineStr">
-        <is>
-          <t>nos</t>
-        </is>
-      </c>
-      <c r="G43" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H43" s="7" t="n"/>
-      <c r="I43" s="8">
-        <f>IF(H43="","",G43*H43)</f>
-        <v/>
-      </c>
-      <c r="J43" s="9" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="10" t="n"/>
-      <c r="B44" s="10" t="inlineStr">
-        <is>
-          <t>Subtotal, section E</t>
-        </is>
-      </c>
-      <c r="C44" s="10" t="n"/>
-      <c r="D44" s="10" t="n"/>
-      <c r="E44" s="10" t="n"/>
-      <c r="F44" s="10" t="n"/>
-      <c r="G44" s="10" t="n"/>
-      <c r="H44" s="10" t="n"/>
-      <c r="I44" s="11">
-        <f>SUM(I41:I43)</f>
-        <v/>
-      </c>
-      <c r="J44" s="10" t="n"/>
-    </row>
-    <row r="46" ht="46" customHeight="1">
-      <c r="A46" s="4" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>Cash and POS</t>
-        </is>
-      </c>
-      <c r="C46" s="4" t="n"/>
-      <c r="D46" s="4" t="n"/>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>At the door end of the back bar, where bills are settled.</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="n"/>
-      <c r="G46" s="4" t="n"/>
-      <c r="H46" s="4" t="n"/>
-      <c r="I46" s="4" t="n"/>
-      <c r="J46" s="4" t="n"/>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>POS nook</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Recessed into the back bar, door end</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>0.48 × 0.40 × 0.96 to 1.35</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Timber frame; room for tablet, card machine and receipt printer</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>nos</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H46" s="7" t="n"/>
+      <c r="I46" s="8">
+        <f>IF(H46="","",G46*H46)</f>
+        <v/>
+      </c>
+      <c r="J46" s="9" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n">
@@ -1769,22 +1769,22 @@
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>POS nook</t>
+          <t>Cash drawer with small safe</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Recessed into the back bar, door end</t>
+          <t>Under the POS nook</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>0.48 × 0.40 × 0.96 to 1.35</t>
+          <t>0.40 × 0.24</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Timber frame; room for tablet, card machine and receipt printer</t>
+          <t>Lockable</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -1803,86 +1803,86 @@
       <c r="J47" s="9" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="n">
+      <c r="A48" s="10" t="n"/>
+      <c r="B48" s="10" t="inlineStr">
+        <is>
+          <t>Subtotal, section F</t>
+        </is>
+      </c>
+      <c r="C48" s="10" t="n"/>
+      <c r="D48" s="10" t="n"/>
+      <c r="E48" s="10" t="n"/>
+      <c r="F48" s="10" t="n"/>
+      <c r="G48" s="10" t="n"/>
+      <c r="H48" s="10" t="n"/>
+      <c r="I48" s="11">
+        <f>SUM(I46:I47)</f>
+        <v/>
+      </c>
+      <c r="J48" s="10" t="n"/>
+    </row>
+    <row r="50" ht="46" customHeight="1">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Server station</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="n"/>
+      <c r="D50" s="4" t="n"/>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>On the left wall just past the back bar, two steps from the kitchen door.</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="n"/>
+      <c r="G50" s="4" t="n"/>
+      <c r="H50" s="4" t="n"/>
+      <c r="I50" s="4" t="n"/>
+      <c r="J50" s="4" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n">
         <v>27</v>
       </c>
-      <c r="B48" s="5" t="inlineStr">
-        <is>
-          <t>Cash drawer with small safe</t>
-        </is>
-      </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>Under the POS nook</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>0.40 × 0.24</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Lockable</t>
-        </is>
-      </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>nos</t>
-        </is>
-      </c>
-      <c r="G48" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H48" s="7" t="n"/>
-      <c r="I48" s="8">
-        <f>IF(H48="","",G48*H48)</f>
-        <v/>
-      </c>
-      <c r="J48" s="9" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="10" t="n"/>
-      <c r="B49" s="10" t="inlineStr">
-        <is>
-          <t>Subtotal, section F</t>
-        </is>
-      </c>
-      <c r="C49" s="10" t="n"/>
-      <c r="D49" s="10" t="n"/>
-      <c r="E49" s="10" t="n"/>
-      <c r="F49" s="10" t="n"/>
-      <c r="G49" s="10" t="n"/>
-      <c r="H49" s="10" t="n"/>
-      <c r="I49" s="11">
-        <f>SUM(I47:I48)</f>
-        <v/>
-      </c>
-      <c r="J49" s="10" t="n"/>
-    </row>
-    <row r="51" ht="46" customHeight="1">
-      <c r="A51" s="4" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>Server station</t>
-        </is>
-      </c>
-      <c r="C51" s="4" t="n"/>
-      <c r="D51" s="4" t="n"/>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>On the left wall just past the back bar, two steps from the kitchen door.</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="n"/>
-      <c r="G51" s="4" t="n"/>
-      <c r="H51" s="4" t="n"/>
-      <c r="I51" s="4" t="n"/>
-      <c r="J51" s="4" t="n"/>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Server station counter</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Left wall, past the back bar</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>0.80 × 0.50 × 0.94</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Black base, olive-wood doors, marble top</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>nos</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" s="7" t="n"/>
+      <c r="I51" s="8">
+        <f>IF(H51="","",G51*H51)</f>
+        <v/>
+      </c>
+      <c r="J51" s="9" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="n">
@@ -1890,22 +1890,22 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Server station counter</t>
+          <t>Wall shelf over the station</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Left wall, past the back bar</t>
+          <t>Above the counter</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>0.80 × 0.50 × 0.94</t>
+          <t>0.80 × 0.30</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Black base, olive-wood doors, marble top</t>
+          <t>At 1.60 and 1.95 m, for glasses and cutlery</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
@@ -1914,7 +1914,7 @@
         </is>
       </c>
       <c r="G52" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H52" s="7" t="n"/>
       <c r="I52" s="8">
@@ -1929,22 +1929,18 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>Wall shelf over the station</t>
+          <t>Coffee batch brewer with 2 jugs</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Above the counter</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>0.80 × 0.30</t>
-        </is>
-      </c>
+          <t>On the station counter</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr"/>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>At 1.60 and 1.95 m, for glasses and cutlery</t>
+          <t>About 12 cups a batch; state make and model</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
@@ -1953,7 +1949,7 @@
         </is>
       </c>
       <c r="G53" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H53" s="7" t="n"/>
       <c r="I53" s="8">
@@ -1968,7 +1964,7 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>Coffee batch brewer with 2 jugs</t>
+          <t>Water dispenser</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
@@ -1979,7 +1975,7 @@
       <c r="D54" s="5" t="inlineStr"/>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>About 12 cups a batch; state make and model</t>
+          <t>Chilled and ambient</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
@@ -2003,7 +1999,7 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>Water dispenser</t>
+          <t>Milk warmer</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
@@ -2014,7 +2010,7 @@
       <c r="D55" s="5" t="inlineStr"/>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Chilled and ambient</t>
+          <t>Small</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
@@ -2033,82 +2029,82 @@
       <c r="J55" s="9" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="n">
+      <c r="A56" s="10" t="n"/>
+      <c r="B56" s="10" t="inlineStr">
+        <is>
+          <t>Subtotal, section G</t>
+        </is>
+      </c>
+      <c r="C56" s="10" t="n"/>
+      <c r="D56" s="10" t="n"/>
+      <c r="E56" s="10" t="n"/>
+      <c r="F56" s="10" t="n"/>
+      <c r="G56" s="10" t="n"/>
+      <c r="H56" s="10" t="n"/>
+      <c r="I56" s="11">
+        <f>SUM(I51:I55)</f>
+        <v/>
+      </c>
+      <c r="J56" s="10" t="n"/>
+    </row>
+    <row r="58" ht="46" customHeight="1">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Services and loose items</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="n"/>
+      <c r="D58" s="4" t="n"/>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>Not a place on the plan: the power, water and drains the bar needs, the lighting, and things the bartender brings.</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="n"/>
+      <c r="G58" s="4" t="n"/>
+      <c r="H58" s="4" t="n"/>
+      <c r="I58" s="4" t="n"/>
+      <c r="J58" s="4" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="n">
         <v>32</v>
       </c>
-      <c r="B56" s="5" t="inlineStr">
-        <is>
-          <t>Milk warmer</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>On the station counter</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr"/>
-      <c r="E56" s="5" t="inlineStr">
-        <is>
-          <t>Small</t>
-        </is>
-      </c>
-      <c r="F56" s="5" t="inlineStr">
-        <is>
-          <t>nos</t>
-        </is>
-      </c>
-      <c r="G56" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H56" s="7" t="n"/>
-      <c r="I56" s="8">
-        <f>IF(H56="","",G56*H56)</f>
-        <v/>
-      </c>
-      <c r="J56" s="9" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="10" t="n"/>
-      <c r="B57" s="10" t="inlineStr">
-        <is>
-          <t>Subtotal, section G</t>
-        </is>
-      </c>
-      <c r="C57" s="10" t="n"/>
-      <c r="D57" s="10" t="n"/>
-      <c r="E57" s="10" t="n"/>
-      <c r="F57" s="10" t="n"/>
-      <c r="G57" s="10" t="n"/>
-      <c r="H57" s="10" t="n"/>
-      <c r="I57" s="11">
-        <f>SUM(I52:I56)</f>
-        <v/>
-      </c>
-      <c r="J57" s="10" t="n"/>
-    </row>
-    <row r="59" ht="46" customHeight="1">
-      <c r="A59" s="4" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="inlineStr">
-        <is>
-          <t>Services and loose items</t>
-        </is>
-      </c>
-      <c r="C59" s="4" t="n"/>
-      <c r="D59" s="4" t="n"/>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>Not a place on the plan: the power, water and drains the bar needs, the lighting, and things the bartender brings.</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="n"/>
-      <c r="G59" s="4" t="n"/>
-      <c r="H59" s="4" t="n"/>
-      <c r="I59" s="4" t="n"/>
-      <c r="J59" s="4" t="n"/>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Power points</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Across the bar and the station</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr"/>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Ice machine, glasswasher, cooler, flash chiller, POS, TV, neon, LED strips, coffee brewer, water dispenser; the chillers and POS on the power backup</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>nos</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="H59" s="7" t="n"/>
+      <c r="I59" s="8">
+        <f>IF(H59="","",G59*H59)</f>
+        <v/>
+      </c>
+      <c r="J59" s="9" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="5" t="n">
@@ -2116,18 +2112,18 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Power points</t>
+          <t>Water points with isolation valves</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Across the bar and the station</t>
+          <t>Bar sink, glasswasher, ice machine, coffee brewer</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr"/>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>Ice machine, glasswasher, cooler, flash chiller, POS, TV, neon, LED strips, coffee brewer, water dispenser; the chillers and POS on the power backup</t>
+          <t>Hot and cold at the sink and glasswasher; filtered cold at the ice machine</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
@@ -2136,7 +2132,7 @@
         </is>
       </c>
       <c r="G60" s="6" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H60" s="7" t="n"/>
       <c r="I60" s="8">
@@ -2151,18 +2147,18 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>Water points with isolation valves</t>
+          <t>Drain points to the grey-water line</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Bar sink, glasswasher, ice machine, coffee brewer</t>
+          <t>Bar sink and ice basin, glasswasher, ice machine</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr"/>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Hot and cold at the sink and glasswasher; filtered cold at the ice machine</t>
+          <t>Never to the biodigester</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
@@ -2186,27 +2182,27 @@
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Drain points to the grey-water line</t>
+          <t>Warm LED strips and downlights</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Bar sink, glasswasher, ice machine, ice well</t>
+          <t>Under both long sides of the counter; 4 over the marble</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr"/>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>Never to the biodigester</t>
+          <t>2,200 K</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>nos</t>
+          <t>lot</t>
         </is>
       </c>
       <c r="G62" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H62" s="7" t="n"/>
       <c r="I62" s="8">
@@ -2221,18 +2217,18 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>Warm LED strips and downlights</t>
+          <t>Bar smallware</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Under both long sides of the counter; 4 over the marble</t>
+          <t>Bartender brings or buys</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr"/>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>2,200 K</t>
+          <t>To the bar consultant's list: shakers, jiggers, strainers, muddlers, bar mats</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
@@ -2256,18 +2252,18 @@
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Bar smallware</t>
+          <t>Glassware</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Bartender brings or buys</t>
+          <t>Per the drinks menu</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr"/>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>To the bar consultant's list: shakers, jiggers, strainers, muddlers, bar mats</t>
+          <t>Pint, gose, whisky, highball, coupe, shot; see the crockery list (breweries often give branded pint glasses)</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
@@ -2286,74 +2282,47 @@
       <c r="J64" s="9" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="5" t="n">
-        <v>38</v>
-      </c>
-      <c r="B65" s="5" t="inlineStr">
-        <is>
-          <t>Glassware</t>
-        </is>
-      </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>Per the drinks menu</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr"/>
-      <c r="E65" s="5" t="inlineStr">
-        <is>
-          <t>Pint, gose, whisky, highball, coupe, shot; see the crockery list (breweries often give branded pint glasses)</t>
-        </is>
-      </c>
-      <c r="F65" s="5" t="inlineStr">
-        <is>
-          <t>lot</t>
-        </is>
-      </c>
-      <c r="G65" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H65" s="7" t="n"/>
-      <c r="I65" s="8">
-        <f>IF(H65="","",G65*H65)</f>
-        <v/>
-      </c>
-      <c r="J65" s="9" t="n"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="10" t="n"/>
-      <c r="B66" s="10" t="inlineStr">
+      <c r="A65" s="10" t="n"/>
+      <c r="B65" s="10" t="inlineStr">
         <is>
           <t>Subtotal, section H</t>
         </is>
       </c>
-      <c r="C66" s="10" t="n"/>
-      <c r="D66" s="10" t="n"/>
-      <c r="E66" s="10" t="n"/>
-      <c r="F66" s="10" t="n"/>
-      <c r="G66" s="10" t="n"/>
-      <c r="H66" s="10" t="n"/>
-      <c r="I66" s="11">
-        <f>SUM(I60:I65)</f>
-        <v/>
-      </c>
-      <c r="J66" s="10" t="n"/>
+      <c r="C65" s="10" t="n"/>
+      <c r="D65" s="10" t="n"/>
+      <c r="E65" s="10" t="n"/>
+      <c r="F65" s="10" t="n"/>
+      <c r="G65" s="10" t="n"/>
+      <c r="H65" s="10" t="n"/>
+      <c r="I65" s="11">
+        <f>SUM(I59:I64)</f>
+        <v/>
+      </c>
+      <c r="J65" s="10" t="n"/>
+    </row>
+    <row r="67">
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>Total of all sections (ex-GST)</t>
+        </is>
+      </c>
+      <c r="I67" s="13">
+        <f>I10+I20+I28+I37+I43+I48+I56+I65</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="B68" s="12" t="inlineStr">
         <is>
-          <t>Total of all sections (ex-GST)</t>
-        </is>
-      </c>
-      <c r="I68" s="13">
-        <f>I10+I20+I29+I38+I44+I49+I57+I66</f>
-        <v/>
-      </c>
+          <t>Freight and unloading to Betalbatim</t>
+        </is>
+      </c>
+      <c r="I68" s="14" t="n"/>
     </row>
     <row r="69">
       <c r="B69" s="12" t="inlineStr">
         <is>
-          <t>Freight and unloading to Betalbatim</t>
+          <t>Installation and connections not included above</t>
         </is>
       </c>
       <c r="I69" s="14" t="n"/>
@@ -2361,40 +2330,32 @@
     <row r="70">
       <c r="B70" s="12" t="inlineStr">
         <is>
-          <t>Installation and connections not included above</t>
-        </is>
-      </c>
-      <c r="I70" s="14" t="n"/>
+          <t>GST rate (%)</t>
+        </is>
+      </c>
+      <c r="I70" s="14" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="71">
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t>GST rate (%)</t>
-        </is>
-      </c>
-      <c r="I71" s="14" t="n">
-        <v>18</v>
+          <t>GST</t>
+        </is>
+      </c>
+      <c r="I71" s="13">
+        <f>ROUND((I67+I68+I69)*I70/100,2)</f>
+        <v/>
       </c>
     </row>
     <row r="72">
-      <c r="B72" s="12" t="inlineStr">
-        <is>
-          <t>GST</t>
-        </is>
-      </c>
-      <c r="I72" s="13">
-        <f>ROUND((I68+I69+I70)*I71/100,2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73">
-      <c r="B73" s="15" t="inlineStr">
+      <c r="B72" s="15" t="inlineStr">
         <is>
           <t>Grand total including GST</t>
         </is>
       </c>
-      <c r="I73" s="16">
-        <f>I68+I69+I70+I72</f>
+      <c r="I72" s="16">
+        <f>I67+I68+I69+I71</f>
         <v/>
       </c>
     </row>

</xml_diff>